<commit_message>
Auto sync Onetech 31/10/2026 08:46
</commit_message>
<xml_diff>
--- a/data/Thang10/DanhSachChiTietDonHang (2).xlsx
+++ b/data/Thang10/DanhSachChiTietDonHang (2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="137">
   <si>
     <t>BÁO CÁO LINE ITEM</t>
   </si>
@@ -151,36 +151,123 @@
     <t>Công Ty TNHH Minh Phát Thành</t>
   </si>
   <si>
+    <t>22SF.HC11949</t>
+  </si>
+  <si>
+    <t>Đinh Ngọc Thông</t>
+  </si>
+  <si>
+    <t>MIX_LE</t>
+  </si>
+  <si>
+    <t>SM-FM-10KF1326.15</t>
+  </si>
+  <si>
+    <t>W-284907920433221</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>DM-10KF1326.01</t>
+  </si>
+  <si>
+    <t>Nguyễn Út Đèo</t>
+  </si>
+  <si>
+    <t>Đơn hàng giao sau</t>
+  </si>
+  <si>
+    <t>Đã gửi đơn</t>
+  </si>
+  <si>
+    <t>31/10/2026 08:35:10</t>
+  </si>
+  <si>
+    <t>2849079</t>
+  </si>
+  <si>
+    <t>Tạp Hóa Nhân Thịnh</t>
+  </si>
+  <si>
+    <t>1017 Nguyễn Duy Trinh</t>
+  </si>
+  <si>
+    <t>Hồ Chí Minh</t>
+  </si>
+  <si>
+    <t>P. Long Trường</t>
+  </si>
+  <si>
+    <t>Beer</t>
+  </si>
+  <si>
+    <t>Bia Red Ruby Cao Cấp</t>
+  </si>
+  <si>
+    <t>08BI00081</t>
+  </si>
+  <si>
+    <t>Bia Red Ruby (sleek) KM TC 24lon x 330ml</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Processed Meats</t>
+  </si>
+  <si>
+    <t>Xúc Xích Cao Bồi Xốt Lắc</t>
+  </si>
+  <si>
+    <t>02XX00223</t>
+  </si>
+  <si>
+    <t>Xúc xích tiệt trùng Heo cao bồi xốt spagetti 48ly x (3cây x 13gr + 1gói xốt 12gr)</t>
+  </si>
+  <si>
+    <t>02XX00224</t>
+  </si>
+  <si>
+    <t>Xúc xích tiệt trùng Heo cao bồi lắc phô mai 48ly x (3cây x 13gr + 1gói lắc 3.2gr)</t>
+  </si>
+  <si>
+    <t>02XX00225</t>
+  </si>
+  <si>
+    <t>Xúc xích tiệt trùng Heo cao bồi xốt tôm sữa 48ly x (3cây x 13gr + 1gói xốt 12gr + 1gói hạt giòn 1.5gr)</t>
+  </si>
+  <si>
+    <t>02XX00226</t>
+  </si>
+  <si>
+    <t>Xúc xích tiệt trùng Heo cao bồi lắc phô mai bắp bơ 48ly x (3cây x 13gr + 1gói lắc 3gr)</t>
+  </si>
+  <si>
+    <t>Seasoning</t>
+  </si>
+  <si>
+    <t>Xốt nhà hàng Chinsu</t>
+  </si>
+  <si>
+    <t>03MR00023</t>
+  </si>
+  <si>
+    <t>Xốt nhà hàng CHIN-SU nướng muối ớt 8hộp x 10túi x 80gr</t>
+  </si>
+  <si>
     <t>26SF.HC22776</t>
   </si>
   <si>
     <t>Nguyễn Tấn Trung</t>
   </si>
   <si>
-    <t>MIX_LE</t>
-  </si>
-  <si>
     <t>SM-FM-10KF1326.43</t>
   </si>
   <si>
     <t>R-132620429854</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>DM-10KF1326.01</t>
-  </si>
-  <si>
-    <t>Nguyễn Út Đèo</t>
-  </si>
-  <si>
-    <t>Đơn hàng giao sau</t>
-  </si>
-  <si>
-    <t>Đã gửi đơn</t>
-  </si>
-  <si>
     <t>31/10/2026 07:52:22</t>
   </si>
   <si>
@@ -193,15 +280,9 @@
     <t>594 Nguyễn Duy Trinh</t>
   </si>
   <si>
-    <t>Hồ Chí Minh</t>
-  </si>
-  <si>
     <t>P. Bình Trưng</t>
   </si>
   <si>
-    <t>Seasoning</t>
-  </si>
-  <si>
     <t>Nước mắm Nam Ngư</t>
   </si>
   <si>
@@ -211,9 +292,6 @@
     <t>Nước mắm Nam Ngư (QR) MN 3bl x 8chai x 500ml</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>03NM00882</t>
   </si>
   <si>
@@ -229,15 +307,6 @@
     <t>Nước chấm Nam Ngư Đệ Nhị (QR) 15chai x 900ml</t>
   </si>
   <si>
-    <t>22SF.HC11949</t>
-  </si>
-  <si>
-    <t>Đinh Ngọc Thông</t>
-  </si>
-  <si>
-    <t>SM-FM-10KF1326.15</t>
-  </si>
-  <si>
     <t>W-261630420429704</t>
   </si>
   <si>
@@ -253,9 +322,6 @@
     <t>1027 Nguyễn Duy Trinh</t>
   </si>
   <si>
-    <t>P. Long Trường</t>
-  </si>
-  <si>
     <t>Nutrition</t>
   </si>
   <si>
@@ -268,36 +334,6 @@
     <t>Sữa hạt ngũ cốc B'fast (QR) 14bịch x 20gói x 25gr</t>
   </si>
   <si>
-    <t>Processed Meats</t>
-  </si>
-  <si>
-    <t>Xúc Xích Cao Bồi Xốt Lắc</t>
-  </si>
-  <si>
-    <t>02XX00223</t>
-  </si>
-  <si>
-    <t>Xúc xích tiệt trùng Heo cao bồi xốt spagetti 48ly x (3cây x 13gr + 1gói xốt 12gr)</t>
-  </si>
-  <si>
-    <t>02XX00224</t>
-  </si>
-  <si>
-    <t>Xúc xích tiệt trùng Heo cao bồi lắc phô mai 48ly x (3cây x 13gr + 1gói lắc 3.2gr)</t>
-  </si>
-  <si>
-    <t>02XX00225</t>
-  </si>
-  <si>
-    <t>Xúc xích tiệt trùng Heo cao bồi xốt tôm sữa 48ly x (3cây x 13gr + 1gói xốt 12gr + 1gói hạt giòn 1.5gr)</t>
-  </si>
-  <si>
-    <t>02XX00226</t>
-  </si>
-  <si>
-    <t>Xúc xích tiệt trùng Heo cao bồi lắc phô mai bắp bơ 48ly x (3cây x 13gr + 1gói lắc 3gr)</t>
-  </si>
-  <si>
     <t>25SF.HC18701</t>
   </si>
   <si>
@@ -365,9 +401,6 @@
   </si>
   <si>
     <t>Nước tương Tam Thái Tử Nhất ca iode 4bl x 6chai x 500ml</t>
-  </si>
-  <si>
-    <t>Xốt nhà hàng Chinsu</t>
   </si>
   <si>
     <t>03MR00045</t>
@@ -806,7 +839,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AM17"/>
+  <dimension ref="A1:AM23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1027,7 +1060,7 @@
         <v>65</v>
       </c>
       <c r="Z5" s="4">
-        <v>31200</v>
+        <v>9583.33334</v>
       </c>
       <c r="AA5" s="4">
         <v>24</v>
@@ -1045,10 +1078,10 @@
         <v>24</v>
       </c>
       <c r="AF5" s="4">
-        <v>15.200000000000045</v>
+        <v>8.50608</v>
       </c>
       <c r="AG5" s="5">
-        <v>748800</v>
+        <v>230000.00016</v>
       </c>
       <c r="AH5" s="5">
         <v>0</v>
@@ -1057,10 +1090,10 @@
         <v>0</v>
       </c>
       <c r="AJ5" s="5">
-        <v>748800</v>
+        <v>230000.00016</v>
       </c>
       <c r="AK5" s="5">
-        <v>748800</v>
+        <v>230000.00016</v>
       </c>
       <c r="AL5" s="4" t="s">
         <v>66</v>
@@ -1134,40 +1167,40 @@
         <v>61</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Z6" s="4">
-        <v>44500</v>
+        <v>8386</v>
       </c>
       <c r="AA6" s="4">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="AB6" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD6" s="4">
-        <v>1</v>
+        <v>0.06</v>
       </c>
       <c r="AE6" s="4">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="AF6" s="4">
-        <v>17.100000000000005</v>
+        <v>0.23625</v>
       </c>
       <c r="AG6" s="5">
-        <v>801000</v>
+        <v>25158</v>
       </c>
       <c r="AH6" s="5">
         <v>0</v>
@@ -1176,10 +1209,10 @@
         <v>0</v>
       </c>
       <c r="AJ6" s="5">
-        <v>801000</v>
+        <v>25158</v>
       </c>
       <c r="AK6" s="5">
-        <v>801000</v>
+        <v>25158</v>
       </c>
       <c r="AL6" s="4" t="s">
         <v>66</v>
@@ -1253,40 +1286,40 @@
         <v>61</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="W7" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="X7" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Y7" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Z7" s="4">
-        <v>22200</v>
+        <v>8386</v>
       </c>
       <c r="AA7" s="4">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="AB7" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AC7" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD7" s="4">
-        <v>2</v>
+        <v>0.06</v>
       </c>
       <c r="AE7" s="4">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="AF7" s="4">
-        <v>33</v>
+        <v>0.207500001</v>
       </c>
       <c r="AG7" s="5">
-        <v>666000</v>
+        <v>25158</v>
       </c>
       <c r="AH7" s="5">
         <v>0</v>
@@ -1295,10 +1328,10 @@
         <v>0</v>
       </c>
       <c r="AJ7" s="5">
-        <v>666000</v>
+        <v>25158</v>
       </c>
       <c r="AK7" s="5">
-        <v>666000</v>
+        <v>25158</v>
       </c>
       <c r="AL7" s="4" t="s">
         <v>66</v>
@@ -1315,19 +1348,19 @@
         <v>45</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>51</v>
@@ -1348,7 +1381,7 @@
         <v>55</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="O8" s="4" t="s">
         <v>51</v>
@@ -1357,67 +1390,67 @@
         <v>51</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="T8" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U8" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="W8" s="4" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="X8" s="4" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="Y8" s="4" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="Z8" s="4">
-        <v>53500</v>
+        <v>8386</v>
       </c>
       <c r="AA8" s="4">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="AB8" s="4">
         <v>0</v>
       </c>
       <c r="AC8" s="4">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="AD8" s="4">
-        <v>0.79</v>
+        <v>0.06</v>
       </c>
       <c r="AE8" s="4">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="AF8" s="4">
-        <v>6.230714285714281</v>
+        <v>0.241875</v>
       </c>
       <c r="AG8" s="5">
-        <v>588500</v>
+        <v>25158</v>
       </c>
       <c r="AH8" s="5">
-        <v>246798</v>
+        <v>0</v>
       </c>
       <c r="AI8" s="4">
         <v>0</v>
       </c>
       <c r="AJ8" s="5">
-        <v>341702</v>
+        <v>25158</v>
       </c>
       <c r="AK8" s="5">
-        <v>341702</v>
+        <v>25158</v>
       </c>
       <c r="AL8" s="4" t="s">
         <v>66</v>
@@ -1434,19 +1467,19 @@
         <v>45</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>51</v>
@@ -1467,7 +1500,7 @@
         <v>55</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="O9" s="4" t="s">
         <v>51</v>
@@ -1476,31 +1509,31 @@
         <v>51</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="R9" s="4" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="T9" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="V9" s="4" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="W9" s="4" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="X9" s="4" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="Y9" s="4" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="Z9" s="4">
         <v>8386</v>
@@ -1521,22 +1554,22 @@
         <v>3</v>
       </c>
       <c r="AF9" s="4">
-        <v>0.23625</v>
+        <v>0.206874999</v>
       </c>
       <c r="AG9" s="5">
         <v>25158</v>
       </c>
       <c r="AH9" s="5">
-        <v>10550</v>
+        <v>0</v>
       </c>
       <c r="AI9" s="4">
         <v>0</v>
       </c>
       <c r="AJ9" s="5">
-        <v>14608</v>
+        <v>25158</v>
       </c>
       <c r="AK9" s="5">
-        <v>14608</v>
+        <v>25158</v>
       </c>
       <c r="AL9" s="4" t="s">
         <v>66</v>
@@ -1553,19 +1586,19 @@
         <v>45</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>51</v>
@@ -1586,7 +1619,7 @@
         <v>55</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="O10" s="4" t="s">
         <v>51</v>
@@ -1595,67 +1628,67 @@
         <v>51</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="R10" s="4" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="T10" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V10" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="W10" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="X10" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y10" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="V10" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="W10" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="X10" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y10" s="4" t="s">
-        <v>90</v>
-      </c>
       <c r="Z10" s="4">
-        <v>8386</v>
+        <v>85000</v>
       </c>
       <c r="AA10" s="4">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="AB10" s="4">
         <v>0</v>
       </c>
       <c r="AC10" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD10" s="4">
-        <v>0.06</v>
+        <v>0.13</v>
       </c>
       <c r="AE10" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AF10" s="4">
-        <v>0.207500001</v>
+        <v>1.3</v>
       </c>
       <c r="AG10" s="5">
-        <v>25158</v>
+        <v>85000</v>
       </c>
       <c r="AH10" s="5">
-        <v>10550</v>
+        <v>0</v>
       </c>
       <c r="AI10" s="4">
         <v>0</v>
       </c>
       <c r="AJ10" s="5">
-        <v>14608</v>
+        <v>85000</v>
       </c>
       <c r="AK10" s="5">
-        <v>14608</v>
+        <v>85000</v>
       </c>
       <c r="AL10" s="4" t="s">
         <v>66</v>
@@ -1672,19 +1705,19 @@
         <v>45</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>51</v>
@@ -1705,7 +1738,7 @@
         <v>55</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="O11" s="4" t="s">
         <v>51</v>
@@ -1714,25 +1747,25 @@
         <v>51</v>
       </c>
       <c r="Q11" s="4" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="R11" s="4" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="T11" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="V11" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="W11" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="X11" s="4" t="s">
         <v>91</v>
@@ -1741,40 +1774,40 @@
         <v>92</v>
       </c>
       <c r="Z11" s="4">
-        <v>8386</v>
+        <v>31200</v>
       </c>
       <c r="AA11" s="4">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="AB11" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC11" s="4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD11" s="4">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AE11" s="4">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="AF11" s="4">
-        <v>0.241875</v>
+        <v>15.200000000000045</v>
       </c>
       <c r="AG11" s="5">
-        <v>25158</v>
+        <v>748800</v>
       </c>
       <c r="AH11" s="5">
-        <v>10550</v>
+        <v>0</v>
       </c>
       <c r="AI11" s="4">
         <v>0</v>
       </c>
       <c r="AJ11" s="5">
-        <v>14608</v>
+        <v>748800</v>
       </c>
       <c r="AK11" s="5">
-        <v>14608</v>
+        <v>748800</v>
       </c>
       <c r="AL11" s="4" t="s">
         <v>66</v>
@@ -1791,19 +1824,19 @@
         <v>45</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>51</v>
@@ -1824,7 +1857,7 @@
         <v>55</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="O12" s="4" t="s">
         <v>51</v>
@@ -1833,25 +1866,25 @@
         <v>51</v>
       </c>
       <c r="Q12" s="4" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="T12" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="V12" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="W12" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="X12" s="4" t="s">
         <v>93</v>
@@ -1860,40 +1893,40 @@
         <v>94</v>
       </c>
       <c r="Z12" s="4">
-        <v>8386</v>
+        <v>44500</v>
       </c>
       <c r="AA12" s="4">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="AB12" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC12" s="4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="4">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AE12" s="4">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="AF12" s="4">
-        <v>0.206874999</v>
+        <v>17.100000000000005</v>
       </c>
       <c r="AG12" s="5">
-        <v>25158</v>
+        <v>801000</v>
       </c>
       <c r="AH12" s="5">
-        <v>10552</v>
+        <v>0</v>
       </c>
       <c r="AI12" s="4">
         <v>0</v>
       </c>
       <c r="AJ12" s="5">
-        <v>14606</v>
+        <v>801000</v>
       </c>
       <c r="AK12" s="5">
-        <v>14606</v>
+        <v>801000</v>
       </c>
       <c r="AL12" s="4" t="s">
         <v>66</v>
@@ -1910,19 +1943,19 @@
         <v>45</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>51</v>
@@ -1943,7 +1976,7 @@
         <v>55</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="O13" s="4" t="s">
         <v>51</v>
@@ -1952,37 +1985,37 @@
         <v>51</v>
       </c>
       <c r="Q13" s="4" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="R13" s="4" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="T13" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U13" s="4" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="V13" s="4" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="W13" s="4" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="X13" s="4" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="Y13" s="4" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="Z13" s="4">
-        <v>8000</v>
+        <v>22200</v>
       </c>
       <c r="AA13" s="4">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="AB13" s="4">
         <v>2</v>
@@ -1994,13 +2027,13 @@
         <v>2</v>
       </c>
       <c r="AE13" s="4">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="AF13" s="4">
-        <v>18.499679999999984</v>
+        <v>33</v>
       </c>
       <c r="AG13" s="5">
-        <v>384000</v>
+        <v>666000</v>
       </c>
       <c r="AH13" s="5">
         <v>0</v>
@@ -2009,10 +2042,10 @@
         <v>0</v>
       </c>
       <c r="AJ13" s="5">
-        <v>384000</v>
+        <v>666000</v>
       </c>
       <c r="AK13" s="5">
-        <v>384000</v>
+        <v>666000</v>
       </c>
       <c r="AL13" s="4" t="s">
         <v>66</v>
@@ -2029,19 +2062,19 @@
         <v>45</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>107</v>
+        <v>46</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>108</v>
+        <v>47</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>109</v>
+        <v>49</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>51</v>
@@ -2062,7 +2095,7 @@
         <v>55</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="O14" s="4" t="s">
         <v>51</v>
@@ -2071,67 +2104,67 @@
         <v>51</v>
       </c>
       <c r="Q14" s="4" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="T14" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U14" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="V14" s="4" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="W14" s="4" t="s">
-        <v>63</v>
+        <v>104</v>
       </c>
       <c r="X14" s="4" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="Y14" s="4" t="s">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="Z14" s="4">
-        <v>44500</v>
+        <v>53500</v>
       </c>
       <c r="AA14" s="4">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="AB14" s="4">
         <v>0</v>
       </c>
       <c r="AC14" s="4">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="AD14" s="4">
-        <v>0.33</v>
+        <v>0.79</v>
       </c>
       <c r="AE14" s="4">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="AF14" s="4">
-        <v>5.700000000000002</v>
+        <v>6.230714285714281</v>
       </c>
       <c r="AG14" s="5">
-        <v>267000</v>
+        <v>588500</v>
       </c>
       <c r="AH14" s="5">
-        <v>0</v>
+        <v>246798</v>
       </c>
       <c r="AI14" s="4">
         <v>0</v>
       </c>
       <c r="AJ14" s="5">
-        <v>267000</v>
+        <v>341702</v>
       </c>
       <c r="AK14" s="5">
-        <v>267000</v>
+        <v>341702</v>
       </c>
       <c r="AL14" s="4" t="s">
         <v>66</v>
@@ -2148,19 +2181,19 @@
         <v>45</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>107</v>
+        <v>46</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>108</v>
+        <v>47</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>109</v>
+        <v>49</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>51</v>
@@ -2181,7 +2214,7 @@
         <v>55</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="O15" s="4" t="s">
         <v>51</v>
@@ -2190,67 +2223,67 @@
         <v>51</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="R15" s="4" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="T15" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U15" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="V15" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="W15" s="4" t="s">
-        <v>115</v>
+        <v>68</v>
       </c>
       <c r="X15" s="4" t="s">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="Y15" s="4" t="s">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="Z15" s="4">
-        <v>17500</v>
+        <v>8386</v>
       </c>
       <c r="AA15" s="4">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="AB15" s="4">
         <v>0</v>
       </c>
       <c r="AC15" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AD15" s="4">
-        <v>0.25</v>
+        <v>0.06</v>
       </c>
       <c r="AE15" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AF15" s="4">
-        <v>3.574999999999996</v>
+        <v>0.23625</v>
       </c>
       <c r="AG15" s="5">
-        <v>105000</v>
+        <v>25158</v>
       </c>
       <c r="AH15" s="5">
-        <v>0</v>
+        <v>10550</v>
       </c>
       <c r="AI15" s="4">
         <v>0</v>
       </c>
       <c r="AJ15" s="5">
-        <v>105000</v>
+        <v>14608</v>
       </c>
       <c r="AK15" s="5">
-        <v>105000</v>
+        <v>14608</v>
       </c>
       <c r="AL15" s="4" t="s">
         <v>66</v>
@@ -2267,19 +2300,19 @@
         <v>45</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>107</v>
+        <v>46</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>108</v>
+        <v>47</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>109</v>
+        <v>49</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>51</v>
@@ -2300,7 +2333,7 @@
         <v>55</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="O16" s="4" t="s">
         <v>51</v>
@@ -2309,67 +2342,67 @@
         <v>51</v>
       </c>
       <c r="Q16" s="4" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="R16" s="4" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="T16" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U16" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="V16" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="W16" s="4" t="s">
-        <v>118</v>
+        <v>68</v>
       </c>
       <c r="X16" s="4" t="s">
-        <v>119</v>
+        <v>71</v>
       </c>
       <c r="Y16" s="4" t="s">
-        <v>120</v>
+        <v>72</v>
       </c>
       <c r="Z16" s="4">
-        <v>68000</v>
+        <v>8386</v>
       </c>
       <c r="AA16" s="4">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="AB16" s="4">
         <v>0</v>
       </c>
       <c r="AC16" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD16" s="4">
-        <v>0.13</v>
+        <v>0.06</v>
       </c>
       <c r="AE16" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AF16" s="4">
-        <v>0.87</v>
+        <v>0.207500001</v>
       </c>
       <c r="AG16" s="5">
-        <v>68000</v>
+        <v>25158</v>
       </c>
       <c r="AH16" s="5">
-        <v>0</v>
+        <v>10550</v>
       </c>
       <c r="AI16" s="4">
         <v>0</v>
       </c>
       <c r="AJ16" s="5">
-        <v>68000</v>
+        <v>14608</v>
       </c>
       <c r="AK16" s="5">
-        <v>68000</v>
+        <v>14608</v>
       </c>
       <c r="AL16" s="4" t="s">
         <v>66</v>
@@ -2386,19 +2419,19 @@
         <v>45</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>107</v>
+        <v>46</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>108</v>
+        <v>47</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>109</v>
+        <v>49</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>51</v>
@@ -2419,7 +2452,7 @@
         <v>55</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="O17" s="4" t="s">
         <v>51</v>
@@ -2428,72 +2461,786 @@
         <v>51</v>
       </c>
       <c r="Q17" s="4" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="R17" s="4" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="T17" s="4" t="s">
         <v>60</v>
       </c>
       <c r="U17" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="V17" s="4" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="W17" s="4" t="s">
-        <v>104</v>
+        <v>68</v>
       </c>
       <c r="X17" s="4" t="s">
-        <v>105</v>
+        <v>73</v>
       </c>
       <c r="Y17" s="4" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="Z17" s="4">
-        <v>8000</v>
+        <v>8386</v>
       </c>
       <c r="AA17" s="4">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="AB17" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC17" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD17" s="4">
-        <v>1</v>
+        <v>0.06</v>
       </c>
       <c r="AE17" s="4">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="AF17" s="4">
-        <v>9.249839999999992</v>
+        <v>0.241875</v>
       </c>
       <c r="AG17" s="5">
-        <v>192000</v>
+        <v>25158</v>
       </c>
       <c r="AH17" s="5">
-        <v>0</v>
+        <v>10550</v>
       </c>
       <c r="AI17" s="4">
         <v>0</v>
       </c>
       <c r="AJ17" s="5">
-        <v>192000</v>
+        <v>14608</v>
       </c>
       <c r="AK17" s="5">
-        <v>192000</v>
+        <v>14608</v>
       </c>
       <c r="AL17" s="4" t="s">
         <v>66</v>
       </c>
       <c r="AM17" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q18" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="R18" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="S18" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="T18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U18" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V18" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W18" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="X18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="Z18" s="4">
+        <v>8386</v>
+      </c>
+      <c r="AA18" s="4">
+        <v>48</v>
+      </c>
+      <c r="AB18" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="4">
+        <v>3</v>
+      </c>
+      <c r="AD18" s="4">
+        <v>0.06</v>
+      </c>
+      <c r="AE18" s="4">
+        <v>3</v>
+      </c>
+      <c r="AF18" s="4">
+        <v>0.206874999</v>
+      </c>
+      <c r="AG18" s="5">
+        <v>25158</v>
+      </c>
+      <c r="AH18" s="5">
+        <v>10552</v>
+      </c>
+      <c r="AI18" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ18" s="5">
+        <v>14606</v>
+      </c>
+      <c r="AK18" s="5">
+        <v>14606</v>
+      </c>
+      <c r="AL18" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM18" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q19" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="R19" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="S19" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="T19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U19" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="V19" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="W19" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="X19" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="Y19" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z19" s="4">
+        <v>8000</v>
+      </c>
+      <c r="AA19" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB19" s="4">
+        <v>2</v>
+      </c>
+      <c r="AC19" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="4">
+        <v>2</v>
+      </c>
+      <c r="AE19" s="4">
+        <v>48</v>
+      </c>
+      <c r="AF19" s="4">
+        <v>18.499679999999984</v>
+      </c>
+      <c r="AG19" s="5">
+        <v>384000</v>
+      </c>
+      <c r="AH19" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ19" s="5">
+        <v>384000</v>
+      </c>
+      <c r="AK19" s="5">
+        <v>384000</v>
+      </c>
+      <c r="AL19" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM19" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q20" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="R20" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="S20" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="T20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U20" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V20" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="W20" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="X20" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="Y20" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z20" s="4">
+        <v>44500</v>
+      </c>
+      <c r="AA20" s="4">
+        <v>18</v>
+      </c>
+      <c r="AB20" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="4">
+        <v>6</v>
+      </c>
+      <c r="AD20" s="4">
+        <v>0.33</v>
+      </c>
+      <c r="AE20" s="4">
+        <v>6</v>
+      </c>
+      <c r="AF20" s="4">
+        <v>5.700000000000002</v>
+      </c>
+      <c r="AG20" s="5">
+        <v>267000</v>
+      </c>
+      <c r="AH20" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI20" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ20" s="5">
+        <v>267000</v>
+      </c>
+      <c r="AK20" s="5">
+        <v>267000</v>
+      </c>
+      <c r="AL20" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM20" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N21" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="O21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q21" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="R21" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="S21" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="T21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U21" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="W21" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="X21" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y21" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="Z21" s="4">
+        <v>17500</v>
+      </c>
+      <c r="AA21" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB21" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="4">
+        <v>6</v>
+      </c>
+      <c r="AD21" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="AE21" s="4">
+        <v>6</v>
+      </c>
+      <c r="AF21" s="4">
+        <v>3.574999999999996</v>
+      </c>
+      <c r="AG21" s="5">
+        <v>105000</v>
+      </c>
+      <c r="AH21" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI21" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ21" s="5">
+        <v>105000</v>
+      </c>
+      <c r="AK21" s="5">
+        <v>105000</v>
+      </c>
+      <c r="AL21" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM21" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M22" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N22" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q22" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="R22" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="S22" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="T22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U22" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V22" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="W22" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="X22" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="Y22" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="Z22" s="4">
+        <v>68000</v>
+      </c>
+      <c r="AA22" s="4">
+        <v>8</v>
+      </c>
+      <c r="AB22" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="4">
+        <v>1</v>
+      </c>
+      <c r="AD22" s="4">
+        <v>0.13</v>
+      </c>
+      <c r="AE22" s="4">
+        <v>1</v>
+      </c>
+      <c r="AF22" s="4">
+        <v>0.87</v>
+      </c>
+      <c r="AG22" s="5">
+        <v>68000</v>
+      </c>
+      <c r="AH22" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI22" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ22" s="5">
+        <v>68000</v>
+      </c>
+      <c r="AK22" s="5">
+        <v>68000</v>
+      </c>
+      <c r="AL22" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM22" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N23" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q23" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="R23" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="S23" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="T23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U23" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V23" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="W23" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="X23" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="Y23" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z23" s="4">
+        <v>8000</v>
+      </c>
+      <c r="AA23" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB23" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC23" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE23" s="4">
+        <v>24</v>
+      </c>
+      <c r="AF23" s="4">
+        <v>9.249839999999992</v>
+      </c>
+      <c r="AG23" s="5">
+        <v>192000</v>
+      </c>
+      <c r="AH23" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI23" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ23" s="5">
+        <v>192000</v>
+      </c>
+      <c r="AK23" s="5">
+        <v>192000</v>
+      </c>
+      <c r="AL23" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM23" s="5">
         <v>0</v>
       </c>
     </row>

</xml_diff>